<commit_message>
Mise à jour des sections (#118)
* MAJ des profils fsh des sections

* MAJ des ids des profils sections CDA

* MAJ ressources CDA section

* MAJ sections FR-Resultats

* Mise à jour des ids des sections + cardinalités des attributs du code e9a0a34f846cec3fa245d44580f306aebaae1739
</commit_message>
<xml_diff>
--- a/fusionSectionsCDA/ig/StructureDefinition-fr-cda-facteurs-de-risque-professionnels-non-code.xlsx
+++ b/fusionSectionsCDA/ig/StructureDefinition-fr-cda-facteurs-de-risque-professionnels-non-code.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1918" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1920" uniqueCount="245">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-16T10:39:58+00:00</t>
+    <t>2026-04-17T08:40:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>IHE-PCC - Hazardous-Working-Conditions-SectionFacteurs de risques professionnels sous forme narrative (section non codée).</t>
+    <t>IHE-PCC - Hazardous-Working-Conditions-SectionFacteurs de risques professionnels sous forme narrative (section non codÃ©e).</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -411,7 +411,7 @@
     <t>iheSectionHazardousWorkingConditions</t>
   </si>
   <si>
-    <t>Conformité IHE-PCC Hazardous-Working-Conditions-Section (IHE-PCC)</t>
+    <t>ConformitÃ© IHE-PCC Hazardous-Working-Conditions-Section (IHE-PCC)</t>
   </si>
   <si>
     <t>Section.templateId:iheSectionHazardousWorkingConditions.nullFlavor</t>
@@ -456,7 +456,7 @@
     <t>frSectionFacteursDeRisqueProfessionnelsNonCode</t>
   </si>
   <si>
-    <t>Conformité FR-Facteurs-de-risque-professionnels-non-code (CI-SIS)</t>
+    <t>ConformitÃ© FR-Facteurs-de-risque-professionnels-non-code (CI-SIS)</t>
   </si>
   <si>
     <t>Section.templateId:frSectionFacteursDeRisqueProfessionnelsNonCode.nullFlavor</t>
@@ -505,10 +505,13 @@
     <t>Section.id</t>
   </si>
   <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Identifiant de la section</t>
+  </si>
+  <si>
     <t>Section.code</t>
-  </si>
-  <si>
-    <t>Y</t>
   </si>
   <si>
     <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/CE
@@ -3788,7 +3791,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" hidden="true">
+    <row r="27">
       <c r="A27" t="s" s="2">
         <v>158</v>
       </c>
@@ -3801,13 +3804,13 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G27" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>74</v>
+        <v>159</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>74</v>
@@ -3818,8 +3821,12 @@
       <c r="K27" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
+      <c r="L27" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="M27" t="s" s="2">
+        <v>160</v>
+      </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -3889,10 +3896,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3906,7 +3913,7 @@
         <v>75</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>74</v>
@@ -3915,13 +3922,13 @@
         <v>74</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -3972,7 +3979,7 @@
         <v>74</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
@@ -3992,10 +3999,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4091,12 +4098,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="30" hidden="true">
+    <row r="30">
       <c r="A30" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4106,13 +4113,13 @@
         <v>62</v>
       </c>
       <c r="F30" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G30" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H30" t="s" s="2">
-        <v>74</v>
+        <v>159</v>
       </c>
       <c r="I30" t="s" s="2">
         <v>74</v>
@@ -4125,7 +4132,7 @@
       </c>
       <c r="L30" s="2"/>
       <c r="M30" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4137,7 +4144,7 @@
         <v>74</v>
       </c>
       <c r="S30" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T30" t="s" s="2">
         <v>74</v>
@@ -4176,7 +4183,7 @@
         <v>74</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>80</v>
@@ -4194,28 +4201,28 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" hidden="true">
+    <row r="31">
       <c r="A31" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E31" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F31" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>74</v>
+        <v>159</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>74</v>
@@ -4228,7 +4235,7 @@
       </c>
       <c r="L31" s="2"/>
       <c r="M31" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4240,7 +4247,7 @@
         <v>74</v>
       </c>
       <c r="S31" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T31" t="s" s="2">
         <v>74</v>
@@ -4279,7 +4286,7 @@
         <v>74</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>80</v>
@@ -4299,17 +4306,17 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E32" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F32" t="s" s="2">
         <v>80</v>
@@ -4331,7 +4338,7 @@
       </c>
       <c r="L32" s="2"/>
       <c r="M32" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4343,7 +4350,7 @@
         <v>74</v>
       </c>
       <c r="S32" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T32" t="s" s="2">
         <v>74</v>
@@ -4382,7 +4389,7 @@
         <v>74</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>80</v>
@@ -4402,17 +4409,17 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E33" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F33" t="s" s="2">
         <v>80</v>
@@ -4434,7 +4441,7 @@
       </c>
       <c r="L33" s="2"/>
       <c r="M33" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -4485,7 +4492,7 @@
         <v>74</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>80</v>
@@ -4503,28 +4510,28 @@
         <v>74</v>
       </c>
     </row>
-    <row r="34" hidden="true">
+    <row r="34">
       <c r="A34" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E34" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F34" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G34" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H34" t="s" s="2">
-        <v>74</v>
+        <v>159</v>
       </c>
       <c r="I34" t="s" s="2">
         <v>74</v>
@@ -4537,7 +4544,7 @@
       </c>
       <c r="L34" s="2"/>
       <c r="M34" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -4549,7 +4556,7 @@
         <v>74</v>
       </c>
       <c r="S34" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="T34" t="s" s="2">
         <v>74</v>
@@ -4588,7 +4595,7 @@
         <v>74</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -4608,10 +4615,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4634,11 +4641,11 @@
         <v>74</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L35" s="2"/>
       <c r="M35" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -4689,7 +4696,7 @@
         <v>74</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
@@ -4709,10 +4716,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4739,7 +4746,7 @@
       </c>
       <c r="L36" s="2"/>
       <c r="M36" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -4790,7 +4797,7 @@
         <v>74</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>80</v>
@@ -4810,17 +4817,17 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E37" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F37" t="s" s="2">
         <v>80</v>
@@ -4838,11 +4845,11 @@
         <v>74</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L37" s="2"/>
       <c r="M37" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -4893,7 +4900,7 @@
         <v>74</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>80</v>
@@ -4913,17 +4920,17 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E38" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F38" t="s" s="2">
         <v>80</v>
@@ -4941,11 +4948,11 @@
         <v>74</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L38" s="2"/>
       <c r="M38" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -4996,7 +5003,7 @@
         <v>74</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
@@ -5016,17 +5023,17 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E39" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F39" t="s" s="2">
         <v>80</v>
@@ -5044,11 +5051,11 @@
         <v>74</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L39" s="2"/>
       <c r="M39" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5099,7 +5106,7 @@
         <v>74</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
@@ -5119,10 +5126,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5136,7 +5143,7 @@
         <v>75</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>74</v>
@@ -5145,13 +5152,13 @@
         <v>74</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5202,7 +5209,7 @@
         <v>74</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
@@ -5222,10 +5229,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5239,7 +5246,7 @@
         <v>75</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>74</v>
@@ -5248,13 +5255,13 @@
         <v>74</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -5305,7 +5312,7 @@
         <v>74</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
@@ -5325,10 +5332,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -5351,7 +5358,7 @@
         <v>74</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L42" s="2"/>
       <c r="M42" s="2"/>
@@ -5404,7 +5411,7 @@
         <v>74</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
@@ -5424,10 +5431,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -5483,25 +5490,25 @@
       </c>
       <c r="Y43" s="2"/>
       <c r="Z43" t="s" s="2">
+        <v>218</v>
+      </c>
+      <c r="AA43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AF43" t="s" s="2">
         <v>217</v>
-      </c>
-      <c r="AA43" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB43" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC43" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD43" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE43" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF43" t="s" s="2">
-        <v>216</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
@@ -5521,10 +5528,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -5547,7 +5554,7 @@
         <v>74</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
@@ -5600,7 +5607,7 @@
         <v>74</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -5620,10 +5627,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -5646,7 +5653,7 @@
         <v>74</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="L45" s="2"/>
       <c r="M45" s="2"/>
@@ -5699,7 +5706,7 @@
         <v>74</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
@@ -5719,10 +5726,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -5745,7 +5752,7 @@
         <v>74</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
@@ -5798,7 +5805,7 @@
         <v>74</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
@@ -5818,10 +5825,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -5844,7 +5851,7 @@
         <v>74</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="L47" s="2"/>
       <c r="M47" s="2"/>
@@ -5897,7 +5904,7 @@
         <v>74</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -5917,10 +5924,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -5943,7 +5950,7 @@
         <v>74</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L48" s="2"/>
       <c r="M48" s="2"/>
@@ -5996,7 +6003,7 @@
         <v>74</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>80</v>
@@ -6016,10 +6023,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6117,10 +6124,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -6218,10 +6225,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -6319,10 +6326,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -6420,10 +6427,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -6523,10 +6530,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -6626,10 +6633,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -6729,10 +6736,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -6832,10 +6839,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -6933,10 +6940,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -6963,7 +6970,7 @@
       </c>
       <c r="L58" s="2"/>
       <c r="M58" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -6972,7 +6979,7 @@
       </c>
       <c r="Q58" s="2"/>
       <c r="R58" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="S58" t="s" s="2">
         <v>74</v>
@@ -7014,7 +7021,7 @@
         <v>74</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>80</v>
@@ -7034,10 +7041,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -7071,49 +7078,49 @@
       </c>
       <c r="Q59" s="2"/>
       <c r="R59" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="S59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="T59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="U59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="V59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="W59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="X59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="Y59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="Z59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE59" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AF59" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="S59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE59" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF59" t="s" s="2">
-        <v>240</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>80</v>
@@ -7133,10 +7140,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -7159,7 +7166,7 @@
         <v>74</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L60" s="2"/>
       <c r="M60" s="2"/>
@@ -7212,7 +7219,7 @@
         <v>74</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>75</v>

</xml_diff>